<commit_message>
data(rugby_urc): 2026-27 round 1 results, round 2 opening lines
Round 1: all 8 results and turnover counts come from the match-centre
scrape. Every side's points reconcile with its tries, conversions and kicks
(16 of 16). The round's stats are stored in data/stats_2026.csv. The
system went 2-1: Dragons +9.5 W, Munster +3.5 L, Bulls -11.5 W.

Round 2: the 8 opening lines come from the entry sheet. On the open, the
picks are Zebre +17.5, Scarlets +2.5 and Ulster +13.5. These are
provisional until the closing lines are in.

The entry sheet is re-exported with the results, and the site is rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -759,12 +759,36 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -799,12 +823,36 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -839,12 +887,36 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -879,12 +951,36 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -919,12 +1015,36 @@
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -948,7 +1068,11 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>-4.5</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
@@ -980,7 +1104,11 @@
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-17.5</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1012,7 +1140,11 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>-5.5</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1044,7 +1176,11 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1076,7 +1212,11 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>-13.5</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1108,7 +1248,11 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>-10.5</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1140,7 +1284,11 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>-5.5</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1172,7 +1320,11 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
@@ -5687,7 +5839,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Turnovers the HOME side won. Needed as well as conceded: a club's margin is its own conceded minus its own won, and in rugby those are separate counts.</t>
+          <t>Turnovers the HOME side won. Recorded for analysis; the model reads turnovers conceded only (home minus away), so a blank here blocks nothing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(rugby_urc): round 2 lines as at Tuesday 29 Sep, before team naming
This loads the Tuesday lines into closing_line. They are the latest lines
available, so the model now runs on them. They are to be overwritten with
the real close once the teams are named. Three lines moved from the open:
Benetton v Connacht -4.5 to -2.5, Cardiff v Zebre -17.5 to -18.5 and
Munster v Bulls -5.5 to -3.5.

The picks are unchanged: Zebre +18.5, Scarlets +2.5 and Ulster +13.5.
Ulster sits on the edge. At Glasgow -13 or shorter, the power factor
flips and it is no longer a bet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1073,7 +1073,11 @@
           <t>-4.5</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
@@ -1109,7 +1113,11 @@
           <t>-17.5</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>-18.5</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
@@ -1145,7 +1153,11 @@
           <t>-5.5</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>-5.5</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
@@ -1181,7 +1193,11 @@
           <t>-2.5</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
@@ -1217,7 +1233,11 @@
           <t>-13.5</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>-13.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
@@ -1253,7 +1273,11 @@
           <t>-10.5</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>-10.5</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
@@ -1289,7 +1313,11 @@
           <t>-5.5</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>-3.5</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
@@ -1325,7 +1353,11 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 2 closing lines, after team naming
These replace Tuesday's lines in closing_line. Five moved:
  Cardiff v Zebre       -18.5 -> -20.5
  Edinburgh v Stormers   -5.5 ->  +1.5
  Glasgow v Ulster      -13.5 -> -14.5
  Lions v Ospreys       -10.5 -> -12.5
  Sharks v Leinster      +7.5 ->  -4.5  (12-point swing to the Sharks)

The picks are unchanged: Zebre +20.5, Scarlets +2.5 and Ulster +14.5.
Ulster is now a point clear of the edge where the power factor flips
(the ratings make Glasgow 13.4-point favourites).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1115,7 +1115,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>-18.5</t>
+          <t>-20.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>-5.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>-13.5</t>
+          <t>-14.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>-10.5</t>
+          <t>-12.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>-4.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 2 lines as at Saturday 3 Oct
These come from a bookmaker screenshot on matchday and replace Thursday's
closes for the five Saturday matches:
  Lions v Ospreys     -12.5 -> -13.5
  Dragons v Scarlets   -2.5 ->  -3.5
  Glasgow v Ulster    -14.5 -> -15.5
  Sharks v Leinster    -4.5 ->  -5.5
  Munster v Bulls      -3.5 ->  -2.5

The picks are unchanged: Scarlets +3.5 and Ulster +15.5 today, and Zebre
+20.5 played on Friday. The book prices the away handicap at 1.80 and the
home at 1.90.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1195,7 +1195,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>-2.5</t>
+          <t>-3.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>-14.5</t>
+          <t>-15.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>-12.5</t>
+          <t>-13.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>-3.5</t>
+          <t>-2.5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>-4.5</t>
+          <t>-5.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 2 results, round 3 opening lines; freeze played lines
Round 2 results and turnovers come from the match-centre scrape. Every
side's points reconcile with its tries and kicks, 16 of 16. The system
went 2-1: Zebre +20.5 W, Scarlets +3.5 L, Ulster +15.5 W. The season so
far is 4-2, +1.8u.

Round 3 has 8 opening lines from the entry sheet. On the open, the only
pick is Ospreys +2.5 at Dragons (System # -3), provisional until the
closes are in.

The returned sheet was an older copy, carrying Thursday's round 2 lines
for the five Saturday matches. Importing it would have overwritten the
matchday lines. entry_sheet.py now keeps a played match's stored line
when the sheet differs, and lists it. --relines applies the sheet's
value anyway, for a genuine correction. Check 13 covers both cases.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1079,12 +1079,36 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1119,12 +1143,36 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1159,12 +1207,36 @@
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1199,12 +1271,36 @@
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1239,12 +1335,36 @@
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1279,12 +1399,36 @@
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1319,12 +1463,36 @@
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1359,12 +1527,36 @@
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1388,7 +1580,11 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1420,7 +1616,11 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>-12.5</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1452,7 +1652,11 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1484,7 +1688,11 @@
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>-21.5</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1516,7 +1724,11 @@
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>-4.5</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1548,7 +1760,11 @@
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>-7.5</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1580,7 +1796,11 @@
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>-4.5</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1612,7 +1832,11 @@
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 3 closing lines
These are the closing lines from the entry sheet, after team naming.
Five moved from the open:
  Glasgow v Connacht  -12.5 ->  -7.5
  Bulls v Lions        -8.5 -> -10.5
  Leinster v Cardiff  -21.5 -> -23.5
  Scarlets v Benetton  -4.5 ->  -5.5
  Stormers v Sharks    -7.5 ->  -8.5

The only pick is still Ospreys +2.5 at Dragons (System # -3).

The sheet was an older copy carrying Thursday's round 2 lines. The new
freeze kept the stored matchday lines for those five played matches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1585,7 +1585,11 @@
           <t>-2.5</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
@@ -1621,7 +1625,11 @@
           <t>-12.5</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>-7.5</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
@@ -1657,7 +1665,11 @@
           <t>-8.5</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>-10.5</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
@@ -1693,7 +1705,11 @@
           <t>-21.5</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>-23.5</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
@@ -1729,7 +1745,11 @@
           <t>-4.5</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>-5.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
@@ -1765,7 +1785,11 @@
           <t>-7.5</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
@@ -1801,7 +1825,11 @@
           <t>-4.5</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>-4.5</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
@@ -1837,7 +1865,11 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 3 results
Round 3's results and turnovers come from the match-centre scrape. Every
side's points reconcile with its tries and kicks, 16 of 16. The system's
one pick, Ospreys +2.5 at Dragons, won 38-31, which matches the
bookmaker's settlement of your two Ospreys bets. The season so far is 5-2,
+2.8u. Your URC bets are 9-3, +EUR 73.62; the system's picks in the same
rounds, at EUR 25, are +EUR 63.64.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -1591,12 +1591,36 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1631,12 +1655,36 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1671,12 +1719,36 @@
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1711,12 +1783,36 @@
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1751,12 +1847,36 @@
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1791,12 +1911,36 @@
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1831,12 +1975,36 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1871,12 +2039,36 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">

</xml_diff>

<commit_message>
data(rugby_urc): round 4 opening lines
Eight opening handicaps for 23-24 October from the entry sheet. The
sheet was an older copy for round 2's closes; those matches are played,
so the stored closing lines were kept.

Provisional picks (System # at the opening line): Cardiff +1.5 (3),
Lions +8.5 (-4), Ulster +18.5 (-4), Ospreys -8.5 (3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -2092,7 +2092,11 @@
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
@@ -2124,7 +2128,11 @@
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>-18.5</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
@@ -2156,7 +2164,11 @@
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
@@ -2188,7 +2200,11 @@
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
@@ -2220,7 +2236,11 @@
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>-18.5</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
@@ -2252,7 +2272,11 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>-15.5</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
@@ -2284,7 +2308,11 @@
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2316,7 +2344,11 @@
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>-21.5</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 4 closing lines
Eight closing handicaps for 23-24 October, after teams were named. The
sheet was again an older copy for round 2's closes; those matches are
played, so the stored lines were kept.

The picks are unchanged from the opening: Cardiff +2.5 (3), Lions +8.5
(-4), Ulster +16.5 (-4), Ospreys -7.5 (3). Connacht v Zebre moved from
0 to -2 as the line went past the power rating; still no bet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -2097,7 +2097,11 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
@@ -2133,7 +2137,11 @@
           <t>-18.5</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>-21.5</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
@@ -2169,7 +2177,11 @@
           <t>-8.5</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
@@ -2205,7 +2217,11 @@
           <t>8.5</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
@@ -2241,7 +2257,11 @@
           <t>-18.5</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>-16.5</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
@@ -2277,7 +2297,11 @@
           <t>-15.5</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>-16.5</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
@@ -2313,7 +2337,11 @@
           <t>-8.5</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>-7.5</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr"/>
@@ -2349,7 +2377,11 @@
           <t>-21.5</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>-22.5</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 4 match-day closing lines
Three closes moved on match day: Cardiff +1.5 (was +2.5), Connacht
-22.5 (was -21.5), Bulls -15.5 (was -16.5). The picks are unchanged:
Cardiff +1.5 (3), Lions +8.5 (-4), Ulster +15.5 (-4), Ospreys -7.5 (3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -2099,7 +2099,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>-21.5</t>
+          <t>-22.5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>-16.5</t>
+          <t>-15.5</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 4 results, round 5 opening lines
Round 4 from the scrape (urc_202601_round04.csv): all 16 team scores
reconcile with their tries, conversions, penalties and drop goals, and
with the 80-minute score. The system went 2-2: Ulster +15.5 and Ospreys
-7.5 covered, Cardiff +1.5 and Lions +8.5 did not. Season 7-4.

Round 5's two-way opening lines from the entry sheet replace the
three-way readings; seven of the eight were within half a point of them.
Picks at the open: Scarlets +21.5 (-4), Sharks +6.5 (-3), Ulster +12.5
(-3). Ulster's rests on the power vote and drops to -1 if the line comes
in to Stormers -10.5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -2103,12 +2103,36 @@
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2143,12 +2167,36 @@
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2183,12 +2231,36 @@
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2223,12 +2295,36 @@
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2263,12 +2359,36 @@
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2303,12 +2423,36 @@
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2343,12 +2487,36 @@
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2383,12 +2551,36 @@
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2414,7 +2606,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
@@ -2450,7 +2642,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>-14.0</t>
+          <t>-14.5</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -2486,7 +2678,7 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -2522,7 +2714,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>-21.0</t>
+          <t>-21.5</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
@@ -2558,7 +2750,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>-10.0</t>
+          <t>-10.5</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -2594,7 +2786,7 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>-6.0</t>
+          <t>-6.5</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
@@ -2630,7 +2822,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>-3.0</t>
+          <t>-3.5</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
@@ -2666,7 +2858,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>-11.0</t>
+          <t>-12.5</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
data(rugby_urc): round 5 closing lines
Eight closing handicaps for 30-31 October, after teams were named. Big
moves on team news: Connacht v Leinster +3.5 -> -3.5, Glasgow v Lions
-14.5 -> -6.5, Bulls -21.5 -> -25.5, Munster -6.5 -> -2.5, Stormers
-12.5 -> -16.5.

The picks are the same three as at the open: Scarlets +25.5 (-4),
Sharks +2.5 (-3), Ulster +16.5 (-3). Ulster's knife edge is gone, as
the line moved away from the power rating. Glasgow v Lions goes 0 -> +2
on the power vote; still no bet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111mdxWwY2QTPDZKaoPvua1
</commit_message>
<xml_diff>
--- a/rugby_urc/entry/urc_2026_entry.xlsx
+++ b/rugby_urc/entry/urc_2026_entry.xlsx
@@ -2609,7 +2609,11 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>-3.5</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2645,7 +2649,11 @@
           <t>-14.5</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>-6.5</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr"/>
@@ -2681,7 +2689,11 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr"/>
@@ -2717,7 +2729,11 @@
           <t>-21.5</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>-25.5</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
@@ -2753,7 +2769,11 @@
           <t>-10.5</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>-12.5</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
@@ -2789,7 +2809,11 @@
           <t>-6.5</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
@@ -2825,7 +2849,11 @@
           <t>-3.5</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>-5.5</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
@@ -2861,7 +2889,11 @@
           <t>-12.5</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>-16.5</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr"/>

</xml_diff>